<commit_message>
f29h85x : all : Pull test reports
- Pull test reports from commit 7175c5ff115c9af4cd4a0d14b242ea5fa4c427f6
from work products repo

Fixes: MCAL-30841

Signed-off-by: Piyush Panditrao <p-panditrao@ti.com>
</commit_message>
<xml_diff>
--- a/docs/Test_Report/Cdd_Ecap/TestPlanExecutionReport.xlsx
+++ b/docs/Test_Report/Cdd_Ecap/TestPlanExecutionReport.xlsx
@@ -18,7 +18,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Test Strategy Compliance'!$A$1:$E$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Test Plan | Execution Report'!$A$1:$U$27</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Test Plan | Execution Report'!$A$1:$U$29</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -43,7 +43,7 @@
       <sz val="16"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -77,11 +77,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FF0000"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="00D9E1F2"/>
       </patternFill>
     </fill>
@@ -104,7 +99,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
@@ -136,13 +131,10 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -724,7 +716,7 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>MCAL-30265</t>
+          <t>MCAL-30831</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -734,7 +726,7 @@
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>2025-04-10 21:49:59.711402-05:00 CDT</t>
+          <t>2025-06-09 06:50:16.458892-05:00 CDT</t>
         </is>
       </c>
     </row>
@@ -811,12 +803,12 @@
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>27</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>0</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
@@ -831,7 +823,7 @@
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>27</t>
         </is>
       </c>
     </row>
@@ -1033,12 +1025,12 @@
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>28</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>0</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
@@ -1053,7 +1045,7 @@
       </c>
       <c r="G8" s="3" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>28</t>
         </is>
       </c>
     </row>
@@ -1124,12 +1116,12 @@
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>88%</t>
+          <t>100%</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>12%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
@@ -1353,7 +1345,7 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C2" s="3" t="n"/>
       <c r="D2" s="3" t="inlineStr">
@@ -1362,7 +1354,7 @@
         </is>
       </c>
       <c r="E2" s="3" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="3">
@@ -1372,7 +1364,7 @@
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C3" s="3" t="n"/>
       <c r="D3" s="3" t="inlineStr">
@@ -1381,7 +1373,7 @@
         </is>
       </c>
       <c r="E3" s="3" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="4">
@@ -1391,7 +1383,7 @@
         </is>
       </c>
       <c r="B4" s="7" t="n">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C4" s="3" t="n"/>
       <c r="D4" s="7" t="inlineStr">
@@ -1400,7 +1392,7 @@
         </is>
       </c>
       <c r="E4" s="7" t="n">
-        <v>26</v>
+        <v>28</v>
       </c>
     </row>
   </sheetData>
@@ -1415,7 +1407,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U27"/>
+  <dimension ref="A1:U29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -1551,22 +1543,22 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>MCAL-30264</t>
+          <t>MCAL-30829</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>F29H85xMCAL_01.02.00: CDD ECAP - Manual Tests</t>
+          <t>F29H85xMCAL_01.02.01: CDD ECAP - Automated Tests</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>MCAL-29917</t>
+          <t>MCAL-30347</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>CDD ECAP Get Version API Test</t>
+          <t>CDD ECAP Set Start Level Condition API Negative Test</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr"/>
@@ -1578,32 +1570,53 @@
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
-          <t>Integration</t>
+          <t>Unit</t>
         </is>
       </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>The test compares the version and print pass in case of match. Anything else is a failure</t>
+          <t>Pass negative parameters to the API and verify right DET errors are generated.</t>
         </is>
       </c>
       <c r="J2" s="3" t="inlineStr">
         <is>
-          <t>&lt;core: c29xx_cpu1&gt;&lt;params_dut:projectid="Cdd_Ecap_Test1";commands=tout:30&gt;</t>
+          <t>{
+  "common_params": {
+    "core_os": [
+      "c29xx_cpu1"
+    ],
+    "test_app_name": "Cdd_Ecap_Test1",
+    "scripts": "generic_mcu_json.py",
+    "no_of_cores": 1,
+    "skip_duplicate": "true",
+    "app_image": {
+      "image_1": {
+        "image_path": "{platform_info.platform}/c29xx_cpu1/c29clang/ram/tests/Cdd_Ecap_Test1/Cdd_Ecap_Test1.out"
+      }
+    },
+    "constraint": {
+      "constraint_1":{
+        "message": "All tests have passed",
+        "port": "mcu0"
+      }
+    }
+  }
+}</t>
         </is>
       </c>
       <c r="K2" s="3" t="inlineStr">
         <is>
-          <t>The test compares the version and print pass in case of match</t>
+          <t>The test passes wrong parameter to the driver. The driver should call DET with expected errors. The UT verifies this and mark the test as a pass. If errors are not created. then this is treated as a failure</t>
         </is>
       </c>
       <c r="L2" s="3" t="inlineStr">
         <is>
-          <t>Functional</t>
+          <t>Interface</t>
         </is>
       </c>
       <c r="M2" s="3" t="inlineStr">
         <is>
-          <t>Requirements-Analysis</t>
+          <t>Boundary Value Analysis</t>
         </is>
       </c>
       <c r="N2" s="3" t="inlineStr">
@@ -1623,12 +1636,12 @@
       </c>
       <c r="Q2" s="3" t="inlineStr">
         <is>
-          <t>MCAL-30265</t>
+          <t>MCAL-30831</t>
         </is>
       </c>
       <c r="R2" s="3" t="inlineStr">
         <is>
-          <t>F29H85xMCAL_01.02.00: CDD ECAP - Manual Test Run</t>
+          <t>F29H85xMCAL_01.02.01: CDD ECAP - Automated Test Run</t>
         </is>
       </c>
       <c r="S2" s="3" t="inlineStr"/>
@@ -1642,22 +1655,22 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>MCAL-30264</t>
+          <t>MCAL-30829</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>F29H85xMCAL_01.02.00: CDD ECAP - Manual Tests</t>
+          <t>F29H85xMCAL_01.02.01: CDD ECAP - Automated Tests</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>MCAL-29920</t>
+          <t>MCAL-30345</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>CDD ECAP DeInit API Negative Test</t>
+          <t>CDD ECAP Get Time Elapsed Period Test</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr"/>
@@ -1674,27 +1687,48 @@
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>Pass negative parameters to the API and verify right DET errors are generated.</t>
+          <t>This test loopbacks a GPIO signal to the ECAP module via external wire and input XBAR. Then toggles the GPIO and calculates the elapsed time - period time.</t>
         </is>
       </c>
       <c r="J3" s="3" t="inlineStr">
         <is>
-          <t>&lt;core: c29xx_cpu1&gt;&lt;params_dut:projectid="Cdd_Ecap_Test1";commands=tout:30&gt;</t>
+          <t>{
+  "common_params": {
+    "core_os": [
+      "c29xx_cpu1"
+    ],
+    "test_app_name": "Cdd_Ecap_Test5",
+    "scripts": "generic_mcu_json.py",
+    "no_of_cores": 1,
+    "skip_duplicate": "true",
+    "app_image": {
+      "image_1": {
+        "image_path": "{platform_info.platform}/c29xx_cpu1/c29clang/ram/tests/Cdd_Ecap_Test5/Cdd_Ecap_Test5.out"
+      }
+    },
+    "constraint": {
+      "constraint_1":{
+        "message": "All tests have passed",
+        "port": "mcu0"
+      }
+    }
+  }
+}</t>
         </is>
       </c>
       <c r="K3" s="3" t="inlineStr">
         <is>
-          <t>The test passes wrong parameter to the driver. The driver should call DET with expected errors. The UT verifies this and mark the test as a pass. If errors are not created. then this is treated as a failure</t>
+          <t>The test checks if elapsed time returned by driver matches expectation for various modes. The test passes if this matches. Anything else or any DET error detection is a failure.</t>
         </is>
       </c>
       <c r="L3" s="3" t="inlineStr">
         <is>
-          <t>Interface</t>
+          <t>Functional</t>
         </is>
       </c>
       <c r="M3" s="3" t="inlineStr">
         <is>
-          <t>Boundary Value Analysis</t>
+          <t>Requirements-Analysis</t>
         </is>
       </c>
       <c r="N3" s="3" t="inlineStr">
@@ -1714,12 +1748,12 @@
       </c>
       <c r="Q3" s="3" t="inlineStr">
         <is>
-          <t>MCAL-30265</t>
+          <t>MCAL-30831</t>
         </is>
       </c>
       <c r="R3" s="3" t="inlineStr">
         <is>
-          <t>F29H85xMCAL_01.02.00: CDD ECAP - Manual Test Run</t>
+          <t>F29H85xMCAL_01.02.01: CDD ECAP - Automated Test Run</t>
         </is>
       </c>
       <c r="S3" s="3" t="inlineStr"/>
@@ -1733,22 +1767,22 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>MCAL-30264</t>
+          <t>MCAL-30829</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>F29H85xMCAL_01.02.00: CDD ECAP - Manual Tests</t>
+          <t>F29H85xMCAL_01.02.01: CDD ECAP - Automated Tests</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>MCAL-30135</t>
+          <t>MCAL-30141</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>CDD ECAP Edge Count Test</t>
+          <t>CDD ECAP Get Duty Cycle Test</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr"/>
@@ -1769,17 +1803,38 @@
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>This test loopbacks a GPIO signal to the ECAP module via external wire and input XBAR. Then toggles the GPIO and detect if the ECAP is able to detect the edges. This tests various scenarios like both edge detect, falling edge detect, rising edge detect with start signal as LOW or HIGH.</t>
+          <t>This test loopbacks a GPIO signal to the ECAP module via external wire and input XBAR. Then toggles the GPIO and calculates the duty cycle.</t>
         </is>
       </c>
       <c r="J4" s="3" t="inlineStr">
         <is>
-          <t>&lt;core: c29xx_cpu1&gt;&lt;params_dut:projectid="Cdd_Ecap_Test1";commands=tout:30&gt;</t>
+          <t>{
+  "common_params": {
+    "core_os": [
+      "c29xx_cpu1"
+    ],
+    "test_app_name": "Cdd_Ecap_Test1",
+    "scripts": "generic_mcu_json.py",
+    "no_of_cores": 1,
+    "skip_duplicate": "true",
+    "app_image": {
+      "image_1": {
+        "image_path": "{platform_info.platform}/c29xx_cpu1/c29clang/ram/tests/Cdd_Ecap_Test1/Cdd_Ecap_Test1.out"
+      }
+    },
+    "constraint": {
+      "constraint_1":{
+        "message": "All tests have passed",
+        "port": "mcu0"
+      }
+    }
+  }
+}</t>
         </is>
       </c>
       <c r="K4" s="3" t="inlineStr">
         <is>
-          <t>The test checks if the edge detected matches the expected edge count for various modes. The test passes if this matches. Anything else or any DET error detection is a failure.</t>
+          <t>The test checks if duty cycle returned by driver matches expectation for various modes. The test passes if this matches. Anything else or any DET error detection is a failure.</t>
         </is>
       </c>
       <c r="L4" s="3" t="inlineStr">
@@ -1809,49 +1864,41 @@
       </c>
       <c r="Q4" s="3" t="inlineStr">
         <is>
-          <t>MCAL-30265</t>
+          <t>MCAL-30831</t>
         </is>
       </c>
       <c r="R4" s="3" t="inlineStr">
         <is>
-          <t>F29H85xMCAL_01.02.00: CDD ECAP - Manual Test Run</t>
-        </is>
-      </c>
-      <c r="S4" s="3" t="inlineStr">
-        <is>
-          <t>MCAL-30149</t>
-        </is>
-      </c>
-      <c r="T4" s="3" t="inlineStr">
-        <is>
-          <t>CDD ECAP: First rising edge not detected/not counted in BOTH_EDGE activation condition</t>
-        </is>
-      </c>
-      <c r="U4" s="11" t="inlineStr">
-        <is>
-          <t>Fail</t>
+          <t>F29H85xMCAL_01.02.01: CDD ECAP - Automated Test Run</t>
+        </is>
+      </c>
+      <c r="S4" s="3" t="inlineStr"/>
+      <c r="T4" s="3" t="inlineStr"/>
+      <c r="U4" s="10" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>MCAL-30264</t>
+          <t>MCAL-30829</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>F29H85xMCAL_01.02.00: CDD ECAP - Manual Tests</t>
+          <t>F29H85xMCAL_01.02.01: CDD ECAP - Automated Tests</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>MCAL-30137</t>
+          <t>MCAL-30140</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>CDD ECAP Edge Detect Interrupt Test</t>
+          <t>CDD ECAP Get Time Elapsed Test</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr"/>
@@ -1872,17 +1919,38 @@
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>This test loopbacks a GPIO signal to the ECAP module via external wire and input XBAR. Then toggles the GPIO and detect if the ECAP is able to detect the edges in interrupt mode by enabling the notification feature. This tests various scenarios like both edge detect, falling edge detect, rising edge detect with start signal as LOW or HIGH.</t>
+          <t>This test loopbacks a GPIO signal to the ECAP module via external wire and input XBAR. Then toggles the GPIO and calculates the elapsed time. This tests various scenarios like period, duty cycle, high time and low time</t>
         </is>
       </c>
       <c r="J5" s="3" t="inlineStr">
         <is>
-          <t>&lt;core: c29xx_cpu1&gt;&lt;params_dut:projectid="Cdd_Ecap_Test1";commands=tout:30&gt;</t>
+          <t>{
+  "common_params": {
+    "core_os": [
+      "c29xx_cpu1"
+    ],
+    "test_app_name": "Cdd_Ecap_Test1",
+    "scripts": "generic_mcu_json.py",
+    "no_of_cores": 1,
+    "skip_duplicate": "true",
+    "app_image": {
+      "image_1": {
+        "image_path": "{platform_info.platform}/c29xx_cpu1/c29clang/ram/tests/Cdd_Ecap_Test1/Cdd_Ecap_Test1.out"
+      }
+    },
+    "constraint": {
+      "constraint_1":{
+        "message": "All tests have passed",
+        "port": "mcu0"
+      }
+    }
+  }
+}</t>
         </is>
       </c>
       <c r="K5" s="3" t="inlineStr">
         <is>
-          <t>The test checks if the edge detected matches the expected edge count for various modes. The test passes if this matches. Anything else or any DET error detection is a failure.</t>
+          <t>The test checks if elapsed time returned by driver matches expectation for various modes. The test passes if this matches. Anything else or any DET error detection is a failure.</t>
         </is>
       </c>
       <c r="L5" s="3" t="inlineStr">
@@ -1912,49 +1980,41 @@
       </c>
       <c r="Q5" s="3" t="inlineStr">
         <is>
-          <t>MCAL-30265</t>
+          <t>MCAL-30831</t>
         </is>
       </c>
       <c r="R5" s="3" t="inlineStr">
         <is>
-          <t>F29H85xMCAL_01.02.00: CDD ECAP - Manual Test Run</t>
-        </is>
-      </c>
-      <c r="S5" s="3" t="inlineStr">
-        <is>
-          <t>MCAL-30149</t>
-        </is>
-      </c>
-      <c r="T5" s="3" t="inlineStr">
-        <is>
-          <t>CDD ECAP: First rising edge not detected/not counted in BOTH_EDGE activation condition</t>
-        </is>
-      </c>
-      <c r="U5" s="11" t="inlineStr">
-        <is>
-          <t>Fail</t>
+          <t>F29H85xMCAL_01.02.01: CDD ECAP - Automated Test Run</t>
+        </is>
+      </c>
+      <c r="S5" s="3" t="inlineStr"/>
+      <c r="T5" s="3" t="inlineStr"/>
+      <c r="U5" s="10" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>MCAL-30264</t>
+          <t>MCAL-30829</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>F29H85xMCAL_01.02.00: CDD ECAP - Manual Tests</t>
+          <t>F29H85xMCAL_01.02.01: CDD ECAP - Automated Tests</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>MCAL-30136</t>
+          <t>MCAL-30137</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>CDD ECAP Edge Detect Polling Test</t>
+          <t>CDD ECAP Edge Detect Interrupt Test</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr"/>
@@ -1975,12 +2035,33 @@
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>This test loopbacks a GPIO signal to the ECAP module via external wire and input XBAR. Then toggles the GPIO and detect if the ECAP is able to detect the edges in polling mode. This tests various scenarios like both edge detect, falling edge detect, rising edge detect with start signal as LOW or HIGH.</t>
+          <t>This test loopbacks a GPIO signal to the ECAP module via external wire and input XBAR. Then toggles the GPIO and detect if the ECAP is able to detect the edges in interrupt mode by enabling the notification feature. This tests various scenarios like both edge detect, falling edge detect, rising edge detect with start signal as LOW or HIGH.</t>
         </is>
       </c>
       <c r="J6" s="3" t="inlineStr">
         <is>
-          <t>&lt;core: c29xx_cpu1&gt;&lt;params_dut:projectid="Cdd_Ecap_Test1";commands=tout:30&gt;</t>
+          <t>{
+  "common_params": {
+    "core_os": [
+      "c29xx_cpu1"
+    ],
+    "test_app_name": "Cdd_Ecap_Test1",
+    "scripts": "generic_mcu_json.py",
+    "no_of_cores": 1,
+    "skip_duplicate": "true",
+    "app_image": {
+      "image_1": {
+        "image_path": "{platform_info.platform}/c29xx_cpu1/c29clang/ram/tests/Cdd_Ecap_Test1/Cdd_Ecap_Test1.out"
+      }
+    },
+    "constraint": {
+      "constraint_1":{
+        "message": "All tests have passed",
+        "port": "mcu0"
+      }
+    }
+  }
+}</t>
         </is>
       </c>
       <c r="K6" s="3" t="inlineStr">
@@ -2015,49 +2096,41 @@
       </c>
       <c r="Q6" s="3" t="inlineStr">
         <is>
-          <t>MCAL-30265</t>
+          <t>MCAL-30831</t>
         </is>
       </c>
       <c r="R6" s="3" t="inlineStr">
         <is>
-          <t>F29H85xMCAL_01.02.00: CDD ECAP - Manual Test Run</t>
-        </is>
-      </c>
-      <c r="S6" s="3" t="inlineStr">
-        <is>
-          <t>MCAL-30149</t>
-        </is>
-      </c>
-      <c r="T6" s="3" t="inlineStr">
-        <is>
-          <t>CDD ECAP: First rising edge not detected/not counted in BOTH_EDGE activation condition</t>
-        </is>
-      </c>
-      <c r="U6" s="11" t="inlineStr">
-        <is>
-          <t>Fail</t>
+          <t>F29H85xMCAL_01.02.01: CDD ECAP - Automated Test Run</t>
+        </is>
+      </c>
+      <c r="S6" s="3" t="inlineStr"/>
+      <c r="T6" s="3" t="inlineStr"/>
+      <c r="U6" s="10" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>MCAL-30264</t>
+          <t>MCAL-30829</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>F29H85xMCAL_01.02.00: CDD ECAP - Manual Tests</t>
+          <t>F29H85xMCAL_01.02.01: CDD ECAP - Automated Tests</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>MCAL-30141</t>
+          <t>MCAL-30136</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>CDD ECAP Get Duty Cycle Test</t>
+          <t>CDD ECAP Edge Detect Polling Test</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr"/>
@@ -2078,17 +2151,38 @@
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>This test loopbacks a GPIO signal to the ECAP module via external wire and input XBAR. Then toggles the GPIO and calculates the duty cycle.</t>
+          <t>This test loopbacks a GPIO signal to the ECAP module via external wire and input XBAR. Then toggles the GPIO and detect if the ECAP is able to detect the edges in polling mode. This tests various scenarios like both edge detect, falling edge detect, rising edge detect with start signal as LOW or HIGH.</t>
         </is>
       </c>
       <c r="J7" s="3" t="inlineStr">
         <is>
-          <t>&lt;core: c29xx_cpu1&gt;&lt;params_dut:projectid="Cdd_Ecap_Test1";commands=tout:30&gt;</t>
+          <t>{
+  "common_params": {
+    "core_os": [
+      "c29xx_cpu1"
+    ],
+    "test_app_name": "Cdd_Ecap_Test1",
+    "scripts": "generic_mcu_json.py",
+    "no_of_cores": 1,
+    "skip_duplicate": "true",
+    "app_image": {
+      "image_1": {
+        "image_path": "{platform_info.platform}/c29xx_cpu1/c29clang/ram/tests/Cdd_Ecap_Test1/Cdd_Ecap_Test1.out"
+      }
+    },
+    "constraint": {
+      "constraint_1":{
+        "message": "All tests have passed",
+        "port": "mcu0"
+      }
+    }
+  }
+}</t>
         </is>
       </c>
       <c r="K7" s="3" t="inlineStr">
         <is>
-          <t>The test checks if duty cycle returned by driver matches expectation for various modes. The test passes if this matches. Anything else or any DET error detection is a failure.</t>
+          <t>The test checks if the edge detected matches the expected edge count for various modes. The test passes if this matches. Anything else or any DET error detection is a failure.</t>
         </is>
       </c>
       <c r="L7" s="3" t="inlineStr">
@@ -2118,12 +2212,12 @@
       </c>
       <c r="Q7" s="3" t="inlineStr">
         <is>
-          <t>MCAL-30265</t>
+          <t>MCAL-30831</t>
         </is>
       </c>
       <c r="R7" s="3" t="inlineStr">
         <is>
-          <t>F29H85xMCAL_01.02.00: CDD ECAP - Manual Test Run</t>
+          <t>F29H85xMCAL_01.02.01: CDD ECAP - Automated Test Run</t>
         </is>
       </c>
       <c r="S7" s="3" t="inlineStr"/>
@@ -2137,22 +2231,22 @@
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>MCAL-30264</t>
+          <t>MCAL-30829</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>F29H85xMCAL_01.02.00: CDD ECAP - Manual Tests</t>
+          <t>F29H85xMCAL_01.02.01: CDD ECAP - Automated Tests</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>MCAL-30140</t>
+          <t>MCAL-30135</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>CDD ECAP Get Time Elapsed Test</t>
+          <t>CDD ECAP Edge Count Test</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr"/>
@@ -2173,17 +2267,38 @@
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>This test loopbacks a GPIO signal to the ECAP module via external wire and input XBAR. Then toggles the GPIO and calculates the elapsed time. This tests various scenarios like period, duty cycle, high time and low time</t>
+          <t>This test loopbacks a GPIO signal to the ECAP module via external wire and input XBAR. Then toggles the GPIO and detect if the ECAP is able to detect the edges. This tests various scenarios like both edge detect, falling edge detect, rising edge detect with start signal as LOW or HIGH.</t>
         </is>
       </c>
       <c r="J8" s="3" t="inlineStr">
         <is>
-          <t>&lt;core: c29xx_cpu1&gt;&lt;params_dut:projectid="Cdd_Ecap_Test1";commands=tout:30&gt;</t>
+          <t>{
+  "common_params": {
+    "core_os": [
+      "c29xx_cpu1"
+    ],
+    "test_app_name": "Cdd_Ecap_Test1",
+    "scripts": "generic_mcu_json.py",
+    "no_of_cores": 1,
+    "skip_duplicate": "true",
+    "app_image": {
+      "image_1": {
+        "image_path": "{platform_info.platform}/c29xx_cpu1/c29clang/ram/tests/Cdd_Ecap_Test1/Cdd_Ecap_Test1.out"
+      }
+    },
+    "constraint": {
+      "constraint_1":{
+        "message": "All tests have passed",
+        "port": "mcu0"
+      }
+    }
+  }
+}</t>
         </is>
       </c>
       <c r="K8" s="3" t="inlineStr">
         <is>
-          <t>The test checks if elapsed time returned by driver matches expectation for various modes. The test passes if this matches. Anything else or any DET error detection is a failure.</t>
+          <t>The test checks if the edge detected matches the expected edge count for various modes. The test passes if this matches. Anything else or any DET error detection is a failure.</t>
         </is>
       </c>
       <c r="L8" s="3" t="inlineStr">
@@ -2213,12 +2328,12 @@
       </c>
       <c r="Q8" s="3" t="inlineStr">
         <is>
-          <t>MCAL-30265</t>
+          <t>MCAL-30831</t>
         </is>
       </c>
       <c r="R8" s="3" t="inlineStr">
         <is>
-          <t>F29H85xMCAL_01.02.00: CDD ECAP - Manual Test Run</t>
+          <t>F29H85xMCAL_01.02.01: CDD ECAP - Automated Test Run</t>
         </is>
       </c>
       <c r="S8" s="3" t="inlineStr"/>
@@ -2232,22 +2347,22 @@
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>MCAL-30264</t>
+          <t>MCAL-30829</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>F29H85xMCAL_01.02.00: CDD ECAP - Manual Tests</t>
+          <t>F29H85xMCAL_01.02.01: CDD ECAP - Automated Tests</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>MCAL-29919</t>
+          <t>MCAL-29939</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>CDD ECAP Init API Negative Test</t>
+          <t>CDD ECAP Get Duty Cycle Values API Negative Test</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr"/>
@@ -2269,7 +2384,28 @@
       </c>
       <c r="J9" s="3" t="inlineStr">
         <is>
-          <t>&lt;core: c29xx_cpu1&gt;&lt;params_dut:projectid="Cdd_Ecap_Test1";commands=tout:30&gt;</t>
+          <t>{
+  "common_params": {
+    "core_os": [
+      "c29xx_cpu1"
+    ],
+    "test_app_name": "Cdd_Ecap_Test1",
+    "scripts": "generic_mcu_json.py",
+    "no_of_cores": 1,
+    "skip_duplicate": "true",
+    "app_image": {
+      "image_1": {
+        "image_path": "{platform_info.platform}/c29xx_cpu1/c29clang/ram/tests/Cdd_Ecap_Test1/Cdd_Ecap_Test1.out"
+      }
+    },
+    "constraint": {
+      "constraint_1":{
+        "message": "All tests have passed",
+        "port": "mcu0"
+      }
+    }
+  }
+}</t>
         </is>
       </c>
       <c r="K9" s="3" t="inlineStr">
@@ -2304,12 +2440,12 @@
       </c>
       <c r="Q9" s="3" t="inlineStr">
         <is>
-          <t>MCAL-30265</t>
+          <t>MCAL-30831</t>
         </is>
       </c>
       <c r="R9" s="3" t="inlineStr">
         <is>
-          <t>F29H85xMCAL_01.02.00: CDD ECAP - Manual Test Run</t>
+          <t>F29H85xMCAL_01.02.01: CDD ECAP - Automated Test Run</t>
         </is>
       </c>
       <c r="S9" s="3" t="inlineStr"/>
@@ -2323,22 +2459,22 @@
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>MCAL-30264</t>
+          <t>MCAL-30829</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>F29H85xMCAL_01.02.00: CDD ECAP - Manual Tests</t>
+          <t>F29H85xMCAL_01.02.01: CDD ECAP - Automated Tests</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>MCAL-29927</t>
+          <t>MCAL-29938</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>CDD ECAP Stop Timestamp API Negative Test</t>
+          <t>CDD ECAP Get Time Elapsed API Negative Test</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr"/>
@@ -2360,7 +2496,28 @@
       </c>
       <c r="J10" s="3" t="inlineStr">
         <is>
-          <t>&lt;core: c29xx_cpu1&gt;&lt;params_dut:projectid="Cdd_Ecap_Test1";commands=tout:30&gt;</t>
+          <t>{
+  "common_params": {
+    "core_os": [
+      "c29xx_cpu1"
+    ],
+    "test_app_name": "Cdd_Ecap_Test1",
+    "scripts": "generic_mcu_json.py",
+    "no_of_cores": 1,
+    "skip_duplicate": "true",
+    "app_image": {
+      "image_1": {
+        "image_path": "{platform_info.platform}/c29xx_cpu1/c29clang/ram/tests/Cdd_Ecap_Test1/Cdd_Ecap_Test1.out"
+      }
+    },
+    "constraint": {
+      "constraint_1":{
+        "message": "All tests have passed",
+        "port": "mcu0"
+      }
+    }
+  }
+}</t>
         </is>
       </c>
       <c r="K10" s="3" t="inlineStr">
@@ -2395,12 +2552,12 @@
       </c>
       <c r="Q10" s="3" t="inlineStr">
         <is>
-          <t>MCAL-30265</t>
+          <t>MCAL-30831</t>
         </is>
       </c>
       <c r="R10" s="3" t="inlineStr">
         <is>
-          <t>F29H85xMCAL_01.02.00: CDD ECAP - Manual Test Run</t>
+          <t>F29H85xMCAL_01.02.01: CDD ECAP - Automated Test Run</t>
         </is>
       </c>
       <c r="S10" s="3" t="inlineStr"/>
@@ -2414,22 +2571,22 @@
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>MCAL-30264</t>
+          <t>MCAL-30829</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>F29H85xMCAL_01.02.00: CDD ECAP - Manual Tests</t>
+          <t>F29H85xMCAL_01.02.01: CDD ECAP - Automated Tests</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>MCAL-29925</t>
+          <t>MCAL-29937</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>CDD ECAP Start Timestamp API Negative Test</t>
+          <t>CDD ECAP Stop Signal Measurement API Negative Test</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr"/>
@@ -2451,7 +2608,28 @@
       </c>
       <c r="J11" s="3" t="inlineStr">
         <is>
-          <t>&lt;core: c29xx_cpu1&gt;&lt;params_dut:projectid="Cdd_Ecap_Test1";commands=tout:30&gt;</t>
+          <t>{
+  "common_params": {
+    "core_os": [
+      "c29xx_cpu1"
+    ],
+    "test_app_name": "Cdd_Ecap_Test1",
+    "scripts": "generic_mcu_json.py",
+    "no_of_cores": 1,
+    "skip_duplicate": "true",
+    "app_image": {
+      "image_1": {
+        "image_path": "{platform_info.platform}/c29xx_cpu1/c29clang/ram/tests/Cdd_Ecap_Test1/Cdd_Ecap_Test1.out"
+      }
+    },
+    "constraint": {
+      "constraint_1":{
+        "message": "All tests have passed",
+        "port": "mcu0"
+      }
+    }
+  }
+}</t>
         </is>
       </c>
       <c r="K11" s="3" t="inlineStr">
@@ -2486,12 +2664,12 @@
       </c>
       <c r="Q11" s="3" t="inlineStr">
         <is>
-          <t>MCAL-30265</t>
+          <t>MCAL-30831</t>
         </is>
       </c>
       <c r="R11" s="3" t="inlineStr">
         <is>
-          <t>F29H85xMCAL_01.02.00: CDD ECAP - Manual Test Run</t>
+          <t>F29H85xMCAL_01.02.01: CDD ECAP - Automated Test Run</t>
         </is>
       </c>
       <c r="S11" s="3" t="inlineStr"/>
@@ -2505,22 +2683,22 @@
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>MCAL-30264</t>
+          <t>MCAL-30829</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>F29H85xMCAL_01.02.00: CDD ECAP - Manual Tests</t>
+          <t>F29H85xMCAL_01.02.01: CDD ECAP - Automated Tests</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>MCAL-29923</t>
+          <t>MCAL-29936</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>CDD ECAP Enable Notification API Negative Test</t>
+          <t>CDD ECAP Start Signal Measurement API Negative Test</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr"/>
@@ -2542,7 +2720,28 @@
       </c>
       <c r="J12" s="3" t="inlineStr">
         <is>
-          <t>&lt;core: c29xx_cpu1&gt;&lt;params_dut:projectid="Cdd_Ecap_Test1";commands=tout:30&gt;</t>
+          <t>{
+  "common_params": {
+    "core_os": [
+      "c29xx_cpu1"
+    ],
+    "test_app_name": "Cdd_Ecap_Test1",
+    "scripts": "generic_mcu_json.py",
+    "no_of_cores": 1,
+    "skip_duplicate": "true",
+    "app_image": {
+      "image_1": {
+        "image_path": "{platform_info.platform}/c29xx_cpu1/c29clang/ram/tests/Cdd_Ecap_Test1/Cdd_Ecap_Test1.out"
+      }
+    },
+    "constraint": {
+      "constraint_1":{
+        "message": "All tests have passed",
+        "port": "mcu0"
+      }
+    }
+  }
+}</t>
         </is>
       </c>
       <c r="K12" s="3" t="inlineStr">
@@ -2577,12 +2776,12 @@
       </c>
       <c r="Q12" s="3" t="inlineStr">
         <is>
-          <t>MCAL-30265</t>
+          <t>MCAL-30831</t>
         </is>
       </c>
       <c r="R12" s="3" t="inlineStr">
         <is>
-          <t>F29H85xMCAL_01.02.00: CDD ECAP - Manual Test Run</t>
+          <t>F29H85xMCAL_01.02.01: CDD ECAP - Automated Test Run</t>
         </is>
       </c>
       <c r="S12" s="3" t="inlineStr"/>
@@ -2596,22 +2795,22 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>MCAL-30264</t>
+          <t>MCAL-30829</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>F29H85xMCAL_01.02.00: CDD ECAP - Manual Tests</t>
+          <t>F29H85xMCAL_01.02.01: CDD ECAP - Automated Tests</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>MCAL-29922</t>
+          <t>MCAL-29934</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>CDD ECAP Disable Notification API Negative Test</t>
+          <t>CDD ECAP Disable Edge Detection API Negative Test</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr"/>
@@ -2633,7 +2832,28 @@
       </c>
       <c r="J13" s="3" t="inlineStr">
         <is>
-          <t>&lt;core: c29xx_cpu1&gt;&lt;params_dut:projectid="Cdd_Ecap_Test1";commands=tout:30&gt;</t>
+          <t>{
+  "common_params": {
+    "core_os": [
+      "c29xx_cpu1"
+    ],
+    "test_app_name": "Cdd_Ecap_Test1",
+    "scripts": "generic_mcu_json.py",
+    "no_of_cores": 1,
+    "skip_duplicate": "true",
+    "app_image": {
+      "image_1": {
+        "image_path": "{platform_info.platform}/c29xx_cpu1/c29clang/ram/tests/Cdd_Ecap_Test1/Cdd_Ecap_Test1.out"
+      }
+    },
+    "constraint": {
+      "constraint_1":{
+        "message": "All tests have passed",
+        "port": "mcu0"
+      }
+    }
+  }
+}</t>
         </is>
       </c>
       <c r="K13" s="3" t="inlineStr">
@@ -2668,12 +2888,12 @@
       </c>
       <c r="Q13" s="3" t="inlineStr">
         <is>
-          <t>MCAL-30265</t>
+          <t>MCAL-30831</t>
         </is>
       </c>
       <c r="R13" s="3" t="inlineStr">
         <is>
-          <t>F29H85xMCAL_01.02.00: CDD ECAP - Manual Test Run</t>
+          <t>F29H85xMCAL_01.02.01: CDD ECAP - Automated Test Run</t>
         </is>
       </c>
       <c r="S13" s="3" t="inlineStr"/>
@@ -2687,22 +2907,22 @@
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>MCAL-30264</t>
+          <t>MCAL-30829</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>F29H85xMCAL_01.02.00: CDD ECAP - Manual Tests</t>
+          <t>F29H85xMCAL_01.02.01: CDD ECAP - Automated Tests</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>MCAL-29918</t>
+          <t>MCAL-29933</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>CDD ECAP Get Version API Negative Test</t>
+          <t>CDD ECAP Enable Edge Detection API Negative Test</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr"/>
@@ -2724,7 +2944,28 @@
       </c>
       <c r="J14" s="3" t="inlineStr">
         <is>
-          <t>&lt;core: c29xx_cpu1&gt;&lt;params_dut:projectid="Cdd_Ecap_Test1";commands=tout:30&gt;</t>
+          <t>{
+  "common_params": {
+    "core_os": [
+      "c29xx_cpu1"
+    ],
+    "test_app_name": "Cdd_Ecap_Test1",
+    "scripts": "generic_mcu_json.py",
+    "no_of_cores": 1,
+    "skip_duplicate": "true",
+    "app_image": {
+      "image_1": {
+        "image_path": "{platform_info.platform}/c29xx_cpu1/c29clang/ram/tests/Cdd_Ecap_Test1/Cdd_Ecap_Test1.out"
+      }
+    },
+    "constraint": {
+      "constraint_1":{
+        "message": "All tests have passed",
+        "port": "mcu0"
+      }
+    }
+  }
+}</t>
         </is>
       </c>
       <c r="K14" s="3" t="inlineStr">
@@ -2759,12 +3000,12 @@
       </c>
       <c r="Q14" s="3" t="inlineStr">
         <is>
-          <t>MCAL-30265</t>
+          <t>MCAL-30831</t>
         </is>
       </c>
       <c r="R14" s="3" t="inlineStr">
         <is>
-          <t>F29H85xMCAL_01.02.00: CDD ECAP - Manual Test Run</t>
+          <t>F29H85xMCAL_01.02.01: CDD ECAP - Automated Test Run</t>
         </is>
       </c>
       <c r="S14" s="3" t="inlineStr"/>
@@ -2778,12 +3019,12 @@
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>MCAL-30264</t>
+          <t>MCAL-30829</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>F29H85xMCAL_01.02.00: CDD ECAP - Manual Tests</t>
+          <t>F29H85xMCAL_01.02.01: CDD ECAP - Automated Tests</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
@@ -2815,7 +3056,28 @@
       </c>
       <c r="J15" s="3" t="inlineStr">
         <is>
-          <t>&lt;core: c29xx_cpu1&gt;&lt;params_dut:projectid="Cdd_Ecap_Test1";commands=tout:30&gt;</t>
+          <t>{
+  "common_params": {
+    "core_os": [
+      "c29xx_cpu1"
+    ],
+    "test_app_name": "Cdd_Ecap_Test1",
+    "scripts": "generic_mcu_json.py",
+    "no_of_cores": 1,
+    "skip_duplicate": "true",
+    "app_image": {
+      "image_1": {
+        "image_path": "{platform_info.platform}/c29xx_cpu1/c29clang/ram/tests/Cdd_Ecap_Test1/Cdd_Ecap_Test1.out"
+      }
+    },
+    "constraint": {
+      "constraint_1":{
+        "message": "All tests have passed",
+        "port": "mcu0"
+      }
+    }
+  }
+}</t>
         </is>
       </c>
       <c r="K15" s="3" t="inlineStr">
@@ -2850,12 +3112,12 @@
       </c>
       <c r="Q15" s="3" t="inlineStr">
         <is>
-          <t>MCAL-30265</t>
+          <t>MCAL-30831</t>
         </is>
       </c>
       <c r="R15" s="3" t="inlineStr">
         <is>
-          <t>F29H85xMCAL_01.02.00: CDD ECAP - Manual Test Run</t>
+          <t>F29H85xMCAL_01.02.01: CDD ECAP - Automated Test Run</t>
         </is>
       </c>
       <c r="S15" s="3" t="inlineStr"/>
@@ -2869,12 +3131,12 @@
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>MCAL-30264</t>
+          <t>MCAL-30829</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>F29H85xMCAL_01.02.00: CDD ECAP - Manual Tests</t>
+          <t>F29H85xMCAL_01.02.01: CDD ECAP - Automated Tests</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
@@ -2906,7 +3168,28 @@
       </c>
       <c r="J16" s="3" t="inlineStr">
         <is>
-          <t>&lt;core: c29xx_cpu1&gt;&lt;params_dut:projectid="Cdd_Ecap_Test1";commands=tout:30&gt;</t>
+          <t>{
+  "common_params": {
+    "core_os": [
+      "c29xx_cpu1"
+    ],
+    "test_app_name": "Cdd_Ecap_Test1",
+    "scripts": "generic_mcu_json.py",
+    "no_of_cores": 1,
+    "skip_duplicate": "true",
+    "app_image": {
+      "image_1": {
+        "image_path": "{platform_info.platform}/c29xx_cpu1/c29clang/ram/tests/Cdd_Ecap_Test1/Cdd_Ecap_Test1.out"
+      }
+    },
+    "constraint": {
+      "constraint_1":{
+        "message": "All tests have passed",
+        "port": "mcu0"
+      }
+    }
+  }
+}</t>
         </is>
       </c>
       <c r="K16" s="3" t="inlineStr">
@@ -2941,12 +3224,12 @@
       </c>
       <c r="Q16" s="3" t="inlineStr">
         <is>
-          <t>MCAL-30265</t>
+          <t>MCAL-30831</t>
         </is>
       </c>
       <c r="R16" s="3" t="inlineStr">
         <is>
-          <t>F29H85xMCAL_01.02.00: CDD ECAP - Manual Test Run</t>
+          <t>F29H85xMCAL_01.02.01: CDD ECAP - Automated Test Run</t>
         </is>
       </c>
       <c r="S16" s="3" t="inlineStr"/>
@@ -2960,22 +3243,22 @@
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>MCAL-30264</t>
+          <t>MCAL-30829</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>F29H85xMCAL_01.02.00: CDD ECAP - Manual Tests</t>
+          <t>F29H85xMCAL_01.02.01: CDD ECAP - Automated Tests</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>MCAL-29933</t>
+          <t>MCAL-29930</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>CDD ECAP Enable Edge Detection API Negative Test</t>
+          <t>CDD ECAP Enable Edge Count API Negative Test</t>
         </is>
       </c>
       <c r="E17" s="3" t="inlineStr"/>
@@ -2997,7 +3280,28 @@
       </c>
       <c r="J17" s="3" t="inlineStr">
         <is>
-          <t>&lt;core: c29xx_cpu1&gt;&lt;params_dut:projectid="Cdd_Ecap_Test1";commands=tout:30&gt;</t>
+          <t>{
+  "common_params": {
+    "core_os": [
+      "c29xx_cpu1"
+    ],
+    "test_app_name": "Cdd_Ecap_Test1",
+    "scripts": "generic_mcu_json.py",
+    "no_of_cores": 1,
+    "skip_duplicate": "true",
+    "app_image": {
+      "image_1": {
+        "image_path": "{platform_info.platform}/c29xx_cpu1/c29clang/ram/tests/Cdd_Ecap_Test1/Cdd_Ecap_Test1.out"
+      }
+    },
+    "constraint": {
+      "constraint_1":{
+        "message": "All tests have passed",
+        "port": "mcu0"
+      }
+    }
+  }
+}</t>
         </is>
       </c>
       <c r="K17" s="3" t="inlineStr">
@@ -3032,12 +3336,12 @@
       </c>
       <c r="Q17" s="3" t="inlineStr">
         <is>
-          <t>MCAL-30265</t>
+          <t>MCAL-30831</t>
         </is>
       </c>
       <c r="R17" s="3" t="inlineStr">
         <is>
-          <t>F29H85xMCAL_01.02.00: CDD ECAP - Manual Test Run</t>
+          <t>F29H85xMCAL_01.02.01: CDD ECAP - Automated Test Run</t>
         </is>
       </c>
       <c r="S17" s="3" t="inlineStr"/>
@@ -3051,12 +3355,12 @@
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>MCAL-30264</t>
+          <t>MCAL-30829</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>F29H85xMCAL_01.02.00: CDD ECAP - Manual Tests</t>
+          <t>F29H85xMCAL_01.02.01: CDD ECAP - Automated Tests</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
@@ -3088,7 +3392,28 @@
       </c>
       <c r="J18" s="3" t="inlineStr">
         <is>
-          <t>&lt;core: c29xx_cpu1&gt;&lt;params_dut:projectid="Cdd_Ecap_Test1";commands=tout:30&gt;</t>
+          <t>{
+  "common_params": {
+    "core_os": [
+      "c29xx_cpu1"
+    ],
+    "test_app_name": "Cdd_Ecap_Test1",
+    "scripts": "generic_mcu_json.py",
+    "no_of_cores": 1,
+    "skip_duplicate": "true",
+    "app_image": {
+      "image_1": {
+        "image_path": "{platform_info.platform}/c29xx_cpu1/c29clang/ram/tests/Cdd_Ecap_Test1/Cdd_Ecap_Test1.out"
+      }
+    },
+    "constraint": {
+      "constraint_1":{
+        "message": "All tests have passed",
+        "port": "mcu0"
+      }
+    }
+  }
+}</t>
         </is>
       </c>
       <c r="K18" s="3" t="inlineStr">
@@ -3123,12 +3448,12 @@
       </c>
       <c r="Q18" s="3" t="inlineStr">
         <is>
-          <t>MCAL-30265</t>
+          <t>MCAL-30831</t>
         </is>
       </c>
       <c r="R18" s="3" t="inlineStr">
         <is>
-          <t>F29H85xMCAL_01.02.00: CDD ECAP - Manual Test Run</t>
+          <t>F29H85xMCAL_01.02.01: CDD ECAP - Automated Test Run</t>
         </is>
       </c>
       <c r="S18" s="3" t="inlineStr"/>
@@ -3142,12 +3467,12 @@
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>MCAL-30264</t>
+          <t>MCAL-30829</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>F29H85xMCAL_01.02.00: CDD ECAP - Manual Tests</t>
+          <t>F29H85xMCAL_01.02.01: CDD ECAP - Automated Tests</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
@@ -3179,7 +3504,28 @@
       </c>
       <c r="J19" s="3" t="inlineStr">
         <is>
-          <t>&lt;core: c29xx_cpu1&gt;&lt;params_dut:projectid="Cdd_Ecap_Test1";commands=tout:30&gt;</t>
+          <t>{
+  "common_params": {
+    "core_os": [
+      "c29xx_cpu1"
+    ],
+    "test_app_name": "Cdd_Ecap_Test1",
+    "scripts": "generic_mcu_json.py",
+    "no_of_cores": 1,
+    "skip_duplicate": "true",
+    "app_image": {
+      "image_1": {
+        "image_path": "{platform_info.platform}/c29xx_cpu1/c29clang/ram/tests/Cdd_Ecap_Test1/Cdd_Ecap_Test1.out"
+      }
+    },
+    "constraint": {
+      "constraint_1":{
+        "message": "All tests have passed",
+        "port": "mcu0"
+      }
+    }
+  }
+}</t>
         </is>
       </c>
       <c r="K19" s="3" t="inlineStr">
@@ -3214,12 +3560,12 @@
       </c>
       <c r="Q19" s="3" t="inlineStr">
         <is>
-          <t>MCAL-30265</t>
+          <t>MCAL-30831</t>
         </is>
       </c>
       <c r="R19" s="3" t="inlineStr">
         <is>
-          <t>F29H85xMCAL_01.02.00: CDD ECAP - Manual Test Run</t>
+          <t>F29H85xMCAL_01.02.01: CDD ECAP - Automated Test Run</t>
         </is>
       </c>
       <c r="S19" s="3" t="inlineStr"/>
@@ -3233,22 +3579,22 @@
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>MCAL-30264</t>
+          <t>MCAL-30829</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>F29H85xMCAL_01.02.00: CDD ECAP - Manual Tests</t>
+          <t>F29H85xMCAL_01.02.01: CDD ECAP - Automated Tests</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>MCAL-29930</t>
+          <t>MCAL-29927</t>
         </is>
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>CDD ECAP Enable Edge Count API Negative Test</t>
+          <t>CDD ECAP Stop Timestamp API Negative Test</t>
         </is>
       </c>
       <c r="E20" s="3" t="inlineStr"/>
@@ -3270,7 +3616,28 @@
       </c>
       <c r="J20" s="3" t="inlineStr">
         <is>
-          <t>&lt;core: c29xx_cpu1&gt;&lt;params_dut:projectid="Cdd_Ecap_Test1";commands=tout:30&gt;</t>
+          <t>{
+  "common_params": {
+    "core_os": [
+      "c29xx_cpu1"
+    ],
+    "test_app_name": "Cdd_Ecap_Test1",
+    "scripts": "generic_mcu_json.py",
+    "no_of_cores": 1,
+    "skip_duplicate": "true",
+    "app_image": {
+      "image_1": {
+        "image_path": "{platform_info.platform}/c29xx_cpu1/c29clang/ram/tests/Cdd_Ecap_Test1/Cdd_Ecap_Test1.out"
+      }
+    },
+    "constraint": {
+      "constraint_1":{
+        "message": "All tests have passed",
+        "port": "mcu0"
+      }
+    }
+  }
+}</t>
         </is>
       </c>
       <c r="K20" s="3" t="inlineStr">
@@ -3305,12 +3672,12 @@
       </c>
       <c r="Q20" s="3" t="inlineStr">
         <is>
-          <t>MCAL-30265</t>
+          <t>MCAL-30831</t>
         </is>
       </c>
       <c r="R20" s="3" t="inlineStr">
         <is>
-          <t>F29H85xMCAL_01.02.00: CDD ECAP - Manual Test Run</t>
+          <t>F29H85xMCAL_01.02.01: CDD ECAP - Automated Test Run</t>
         </is>
       </c>
       <c r="S20" s="3" t="inlineStr"/>
@@ -3324,22 +3691,22 @@
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>MCAL-30264</t>
+          <t>MCAL-30829</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>F29H85xMCAL_01.02.00: CDD ECAP - Manual Tests</t>
+          <t>F29H85xMCAL_01.02.01: CDD ECAP - Automated Tests</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>MCAL-29924</t>
+          <t>MCAL-29925</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>CDD ECAP Get Input State API Negative Test</t>
+          <t>CDD ECAP Start Timestamp API Negative Test</t>
         </is>
       </c>
       <c r="E21" s="3" t="inlineStr"/>
@@ -3361,7 +3728,28 @@
       </c>
       <c r="J21" s="3" t="inlineStr">
         <is>
-          <t>&lt;core: c29xx_cpu1&gt;&lt;params_dut:projectid="Cdd_Ecap_Test1";commands=tout:30&gt;</t>
+          <t>{
+  "common_params": {
+    "core_os": [
+      "c29xx_cpu1"
+    ],
+    "test_app_name": "Cdd_Ecap_Test1",
+    "scripts": "generic_mcu_json.py",
+    "no_of_cores": 1,
+    "skip_duplicate": "true",
+    "app_image": {
+      "image_1": {
+        "image_path": "{platform_info.platform}/c29xx_cpu1/c29clang/ram/tests/Cdd_Ecap_Test1/Cdd_Ecap_Test1.out"
+      }
+    },
+    "constraint": {
+      "constraint_1":{
+        "message": "All tests have passed",
+        "port": "mcu0"
+      }
+    }
+  }
+}</t>
         </is>
       </c>
       <c r="K21" s="3" t="inlineStr">
@@ -3396,12 +3784,12 @@
       </c>
       <c r="Q21" s="3" t="inlineStr">
         <is>
-          <t>MCAL-30265</t>
+          <t>MCAL-30831</t>
         </is>
       </c>
       <c r="R21" s="3" t="inlineStr">
         <is>
-          <t>F29H85xMCAL_01.02.00: CDD ECAP - Manual Test Run</t>
+          <t>F29H85xMCAL_01.02.01: CDD ECAP - Automated Test Run</t>
         </is>
       </c>
       <c r="S21" s="3" t="inlineStr"/>
@@ -3415,22 +3803,22 @@
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>MCAL-30264</t>
+          <t>MCAL-30829</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>F29H85xMCAL_01.02.00: CDD ECAP - Manual Tests</t>
+          <t>F29H85xMCAL_01.02.01: CDD ECAP - Automated Tests</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>MCAL-29936</t>
+          <t>MCAL-29924</t>
         </is>
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>CDD ECAP Start Signal Measurement API Negative Test</t>
+          <t>CDD ECAP Get Input State API Negative Test</t>
         </is>
       </c>
       <c r="E22" s="3" t="inlineStr"/>
@@ -3452,7 +3840,28 @@
       </c>
       <c r="J22" s="3" t="inlineStr">
         <is>
-          <t>&lt;core: c29xx_cpu1&gt;&lt;params_dut:projectid="Cdd_Ecap_Test1";commands=tout:30&gt;</t>
+          <t>{
+  "common_params": {
+    "core_os": [
+      "c29xx_cpu1"
+    ],
+    "test_app_name": "Cdd_Ecap_Test1",
+    "scripts": "generic_mcu_json.py",
+    "no_of_cores": 1,
+    "skip_duplicate": "true",
+    "app_image": {
+      "image_1": {
+        "image_path": "{platform_info.platform}/c29xx_cpu1/c29clang/ram/tests/Cdd_Ecap_Test1/Cdd_Ecap_Test1.out"
+      }
+    },
+    "constraint": {
+      "constraint_1":{
+        "message": "All tests have passed",
+        "port": "mcu0"
+      }
+    }
+  }
+}</t>
         </is>
       </c>
       <c r="K22" s="3" t="inlineStr">
@@ -3487,12 +3896,12 @@
       </c>
       <c r="Q22" s="3" t="inlineStr">
         <is>
-          <t>MCAL-30265</t>
+          <t>MCAL-30831</t>
         </is>
       </c>
       <c r="R22" s="3" t="inlineStr">
         <is>
-          <t>F29H85xMCAL_01.02.00: CDD ECAP - Manual Test Run</t>
+          <t>F29H85xMCAL_01.02.01: CDD ECAP - Automated Test Run</t>
         </is>
       </c>
       <c r="S22" s="3" t="inlineStr"/>
@@ -3506,22 +3915,22 @@
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>MCAL-30264</t>
+          <t>MCAL-30829</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>F29H85xMCAL_01.02.00: CDD ECAP - Manual Tests</t>
+          <t>F29H85xMCAL_01.02.01: CDD ECAP - Automated Tests</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>MCAL-29934</t>
+          <t>MCAL-29923</t>
         </is>
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>CDD ECAP Disable Edge Detection API Negative Test</t>
+          <t>CDD ECAP Enable Notification API Negative Test</t>
         </is>
       </c>
       <c r="E23" s="3" t="inlineStr"/>
@@ -3543,7 +3952,28 @@
       </c>
       <c r="J23" s="3" t="inlineStr">
         <is>
-          <t>&lt;core: c29xx_cpu1&gt;&lt;params_dut:projectid="Cdd_Ecap_Test1";commands=tout:30&gt;</t>
+          <t>{
+  "common_params": {
+    "core_os": [
+      "c29xx_cpu1"
+    ],
+    "test_app_name": "Cdd_Ecap_Test1",
+    "scripts": "generic_mcu_json.py",
+    "no_of_cores": 1,
+    "skip_duplicate": "true",
+    "app_image": {
+      "image_1": {
+        "image_path": "{platform_info.platform}/c29xx_cpu1/c29clang/ram/tests/Cdd_Ecap_Test1/Cdd_Ecap_Test1.out"
+      }
+    },
+    "constraint": {
+      "constraint_1":{
+        "message": "All tests have passed",
+        "port": "mcu0"
+      }
+    }
+  }
+}</t>
         </is>
       </c>
       <c r="K23" s="3" t="inlineStr">
@@ -3578,12 +4008,12 @@
       </c>
       <c r="Q23" s="3" t="inlineStr">
         <is>
-          <t>MCAL-30265</t>
+          <t>MCAL-30831</t>
         </is>
       </c>
       <c r="R23" s="3" t="inlineStr">
         <is>
-          <t>F29H85xMCAL_01.02.00: CDD ECAP - Manual Test Run</t>
+          <t>F29H85xMCAL_01.02.01: CDD ECAP - Automated Test Run</t>
         </is>
       </c>
       <c r="S23" s="3" t="inlineStr"/>
@@ -3597,22 +4027,22 @@
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>MCAL-30264</t>
+          <t>MCAL-30829</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>F29H85xMCAL_01.02.00: CDD ECAP - Manual Tests</t>
+          <t>F29H85xMCAL_01.02.01: CDD ECAP - Automated Tests</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>MCAL-29938</t>
+          <t>MCAL-29922</t>
         </is>
       </c>
       <c r="D24" s="3" t="inlineStr">
         <is>
-          <t>CDD ECAP Get Time Elapsed API Negative Test</t>
+          <t>CDD ECAP Disable Notification API Negative Test</t>
         </is>
       </c>
       <c r="E24" s="3" t="inlineStr"/>
@@ -3634,7 +4064,28 @@
       </c>
       <c r="J24" s="3" t="inlineStr">
         <is>
-          <t>&lt;core: c29xx_cpu1&gt;&lt;params_dut:projectid="Cdd_Ecap_Test1";commands=tout:30&gt;</t>
+          <t>{
+  "common_params": {
+    "core_os": [
+      "c29xx_cpu1"
+    ],
+    "test_app_name": "Cdd_Ecap_Test1",
+    "scripts": "generic_mcu_json.py",
+    "no_of_cores": 1,
+    "skip_duplicate": "true",
+    "app_image": {
+      "image_1": {
+        "image_path": "{platform_info.platform}/c29xx_cpu1/c29clang/ram/tests/Cdd_Ecap_Test1/Cdd_Ecap_Test1.out"
+      }
+    },
+    "constraint": {
+      "constraint_1":{
+        "message": "All tests have passed",
+        "port": "mcu0"
+      }
+    }
+  }
+}</t>
         </is>
       </c>
       <c r="K24" s="3" t="inlineStr">
@@ -3669,12 +4120,12 @@
       </c>
       <c r="Q24" s="3" t="inlineStr">
         <is>
-          <t>MCAL-30265</t>
+          <t>MCAL-30831</t>
         </is>
       </c>
       <c r="R24" s="3" t="inlineStr">
         <is>
-          <t>F29H85xMCAL_01.02.00: CDD ECAP - Manual Test Run</t>
+          <t>F29H85xMCAL_01.02.01: CDD ECAP - Automated Test Run</t>
         </is>
       </c>
       <c r="S24" s="3" t="inlineStr"/>
@@ -3688,22 +4139,22 @@
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>MCAL-30264</t>
+          <t>MCAL-30829</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>F29H85xMCAL_01.02.00: CDD ECAP - Manual Tests</t>
+          <t>F29H85xMCAL_01.02.01: CDD ECAP - Automated Tests</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>MCAL-29937</t>
+          <t>MCAL-29921</t>
         </is>
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t>CDD ECAP Stop Signal Measurement API Negative Test</t>
+          <t>CDD ECAP Set Activation Condition API Negative Test</t>
         </is>
       </c>
       <c r="E25" s="3" t="inlineStr"/>
@@ -3725,7 +4176,28 @@
       </c>
       <c r="J25" s="3" t="inlineStr">
         <is>
-          <t>&lt;core: c29xx_cpu1&gt;&lt;params_dut:projectid="Cdd_Ecap_Test1";commands=tout:30&gt;</t>
+          <t>{
+  "common_params": {
+    "core_os": [
+      "c29xx_cpu1"
+    ],
+    "test_app_name": "Cdd_Ecap_Test1",
+    "scripts": "generic_mcu_json.py",
+    "no_of_cores": 1,
+    "skip_duplicate": "true",
+    "app_image": {
+      "image_1": {
+        "image_path": "{platform_info.platform}/c29xx_cpu1/c29clang/ram/tests/Cdd_Ecap_Test1/Cdd_Ecap_Test1.out"
+      }
+    },
+    "constraint": {
+      "constraint_1":{
+        "message": "All tests have passed",
+        "port": "mcu0"
+      }
+    }
+  }
+}</t>
         </is>
       </c>
       <c r="K25" s="3" t="inlineStr">
@@ -3760,12 +4232,12 @@
       </c>
       <c r="Q25" s="3" t="inlineStr">
         <is>
-          <t>MCAL-30265</t>
+          <t>MCAL-30831</t>
         </is>
       </c>
       <c r="R25" s="3" t="inlineStr">
         <is>
-          <t>F29H85xMCAL_01.02.00: CDD ECAP - Manual Test Run</t>
+          <t>F29H85xMCAL_01.02.01: CDD ECAP - Automated Test Run</t>
         </is>
       </c>
       <c r="S25" s="3" t="inlineStr"/>
@@ -3779,22 +4251,22 @@
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t>MCAL-30264</t>
+          <t>MCAL-30829</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>F29H85xMCAL_01.02.00: CDD ECAP - Manual Tests</t>
+          <t>F29H85xMCAL_01.02.01: CDD ECAP - Automated Tests</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>MCAL-29921</t>
+          <t>MCAL-29920</t>
         </is>
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>CDD ECAP Set Activation Condition API Negative Test</t>
+          <t>CDD ECAP DeInit API Negative Test</t>
         </is>
       </c>
       <c r="E26" s="3" t="inlineStr"/>
@@ -3816,7 +4288,28 @@
       </c>
       <c r="J26" s="3" t="inlineStr">
         <is>
-          <t>&lt;core: c29xx_cpu1&gt;&lt;params_dut:projectid="Cdd_Ecap_Test1";commands=tout:30&gt;</t>
+          <t>{
+  "common_params": {
+    "core_os": [
+      "c29xx_cpu1"
+    ],
+    "test_app_name": "Cdd_Ecap_Test1",
+    "scripts": "generic_mcu_json.py",
+    "no_of_cores": 1,
+    "skip_duplicate": "true",
+    "app_image": {
+      "image_1": {
+        "image_path": "{platform_info.platform}/c29xx_cpu1/c29clang/ram/tests/Cdd_Ecap_Test1/Cdd_Ecap_Test1.out"
+      }
+    },
+    "constraint": {
+      "constraint_1":{
+        "message": "All tests have passed",
+        "port": "mcu0"
+      }
+    }
+  }
+}</t>
         </is>
       </c>
       <c r="K26" s="3" t="inlineStr">
@@ -3851,12 +4344,12 @@
       </c>
       <c r="Q26" s="3" t="inlineStr">
         <is>
-          <t>MCAL-30265</t>
+          <t>MCAL-30831</t>
         </is>
       </c>
       <c r="R26" s="3" t="inlineStr">
         <is>
-          <t>F29H85xMCAL_01.02.00: CDD ECAP - Manual Test Run</t>
+          <t>F29H85xMCAL_01.02.01: CDD ECAP - Automated Test Run</t>
         </is>
       </c>
       <c r="S26" s="3" t="inlineStr"/>
@@ -3870,22 +4363,22 @@
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>MCAL-30264</t>
+          <t>MCAL-30829</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>F29H85xMCAL_01.02.00: CDD ECAP - Manual Tests</t>
+          <t>F29H85xMCAL_01.02.01: CDD ECAP - Automated Tests</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>MCAL-29939</t>
+          <t>MCAL-29919</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>CDD ECAP Get Duty Cycle Values API Negative Test</t>
+          <t>CDD ECAP Init API Negative Test</t>
         </is>
       </c>
       <c r="E27" s="3" t="inlineStr"/>
@@ -3907,7 +4400,28 @@
       </c>
       <c r="J27" s="3" t="inlineStr">
         <is>
-          <t>&lt;core: c29xx_cpu1&gt;&lt;params_dut:projectid="Cdd_Ecap_Test1";commands=tout:30&gt;</t>
+          <t>{
+  "common_params": {
+    "core_os": [
+      "c29xx_cpu1"
+    ],
+    "test_app_name": "Cdd_Ecap_Test1",
+    "scripts": "generic_mcu_json.py",
+    "no_of_cores": 1,
+    "skip_duplicate": "true",
+    "app_image": {
+      "image_1": {
+        "image_path": "{platform_info.platform}/c29xx_cpu1/c29clang/ram/tests/Cdd_Ecap_Test1/Cdd_Ecap_Test1.out"
+      }
+    },
+    "constraint": {
+      "constraint_1":{
+        "message": "All tests have passed",
+        "port": "mcu0"
+      }
+    }
+  }
+}</t>
         </is>
       </c>
       <c r="K27" s="3" t="inlineStr">
@@ -3942,12 +4456,12 @@
       </c>
       <c r="Q27" s="3" t="inlineStr">
         <is>
-          <t>MCAL-30265</t>
+          <t>MCAL-30831</t>
         </is>
       </c>
       <c r="R27" s="3" t="inlineStr">
         <is>
-          <t>F29H85xMCAL_01.02.00: CDD ECAP - Manual Test Run</t>
+          <t>F29H85xMCAL_01.02.01: CDD ECAP - Automated Test Run</t>
         </is>
       </c>
       <c r="S27" s="3" t="inlineStr"/>
@@ -3958,8 +4472,232 @@
         </is>
       </c>
     </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>MCAL-30829</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>F29H85xMCAL_01.02.01: CDD ECAP - Automated Tests</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>MCAL-29918</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>CDD ECAP Get Version API Negative Test</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="inlineStr"/>
+      <c r="F28" s="3" t="inlineStr"/>
+      <c r="G28" s="3" t="inlineStr">
+        <is>
+          <t>F29H85x-evm,F29P58x-evm</t>
+        </is>
+      </c>
+      <c r="H28" s="3" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+      <c r="I28" s="3" t="inlineStr">
+        <is>
+          <t>Pass negative parameters to the API and verify right DET errors are generated.</t>
+        </is>
+      </c>
+      <c r="J28" s="3" t="inlineStr">
+        <is>
+          <t>{
+  "common_params": {
+    "core_os": [
+      "c29xx_cpu1"
+    ],
+    "test_app_name": "Cdd_Ecap_Test1",
+    "scripts": "generic_mcu_json.py",
+    "no_of_cores": 1,
+    "skip_duplicate": "true",
+    "app_image": {
+      "image_1": {
+        "image_path": "{platform_info.platform}/c29xx_cpu1/c29clang/ram/tests/Cdd_Ecap_Test1/Cdd_Ecap_Test1.out"
+      }
+    },
+    "constraint": {
+      "constraint_1":{
+        "message": "All tests have passed",
+        "port": "mcu0"
+      }
+    }
+  }
+}</t>
+        </is>
+      </c>
+      <c r="K28" s="3" t="inlineStr">
+        <is>
+          <t>The test passes wrong parameter to the driver. The driver should call DET with expected errors. The UT verifies this and mark the test as a pass. If errors are not created. then this is treated as a failure</t>
+        </is>
+      </c>
+      <c r="L28" s="3" t="inlineStr">
+        <is>
+          <t>Interface</t>
+        </is>
+      </c>
+      <c r="M28" s="3" t="inlineStr">
+        <is>
+          <t>Boundary Value Analysis</t>
+        </is>
+      </c>
+      <c r="N28" s="3" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="O28" s="3" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+      <c r="P28" s="3" t="inlineStr">
+        <is>
+          <t>CDD ECAP</t>
+        </is>
+      </c>
+      <c r="Q28" s="3" t="inlineStr">
+        <is>
+          <t>MCAL-30831</t>
+        </is>
+      </c>
+      <c r="R28" s="3" t="inlineStr">
+        <is>
+          <t>F29H85xMCAL_01.02.01: CDD ECAP - Automated Test Run</t>
+        </is>
+      </c>
+      <c r="S28" s="3" t="inlineStr"/>
+      <c r="T28" s="3" t="inlineStr"/>
+      <c r="U28" s="10" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>MCAL-30829</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>F29H85xMCAL_01.02.01: CDD ECAP - Automated Tests</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>MCAL-29917</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>CDD ECAP Get Version API Test</t>
+        </is>
+      </c>
+      <c r="E29" s="3" t="inlineStr"/>
+      <c r="F29" s="3" t="inlineStr"/>
+      <c r="G29" s="3" t="inlineStr">
+        <is>
+          <t>F29H85x-evm,F29P58x-evm</t>
+        </is>
+      </c>
+      <c r="H29" s="3" t="inlineStr">
+        <is>
+          <t>Integration</t>
+        </is>
+      </c>
+      <c r="I29" s="3" t="inlineStr">
+        <is>
+          <t>The test compares the version and print pass in case of match. Anything else is a failure</t>
+        </is>
+      </c>
+      <c r="J29" s="3" t="inlineStr">
+        <is>
+          <t>{
+  "common_params": {
+    "core_os": [
+      "c29xx_cpu1"
+    ],
+    "test_app_name": "Cdd_Ecap_Test1",
+    "scripts": "generic_mcu_json.py",
+    "no_of_cores": 1,
+    "skip_duplicate": "true",
+    "app_image": {
+      "image_1": {
+        "image_path": "{platform_info.platform}/c29xx_cpu1/c29clang/ram/tests/Cdd_Ecap_Test1/Cdd_Ecap_Test1.out"
+      }
+    },
+    "constraint": {
+      "constraint_1":{
+        "message": "All tests have passed",
+        "port": "mcu0"
+      }
+    }
+  }
+}</t>
+        </is>
+      </c>
+      <c r="K29" s="3" t="inlineStr">
+        <is>
+          <t>The test compares the version and print pass in case of match</t>
+        </is>
+      </c>
+      <c r="L29" s="3" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="M29" s="3" t="inlineStr">
+        <is>
+          <t>Requirements-Analysis</t>
+        </is>
+      </c>
+      <c r="N29" s="3" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="O29" s="3" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+      <c r="P29" s="3" t="inlineStr">
+        <is>
+          <t>CDD ECAP</t>
+        </is>
+      </c>
+      <c r="Q29" s="3" t="inlineStr">
+        <is>
+          <t>MCAL-30831</t>
+        </is>
+      </c>
+      <c r="R29" s="3" t="inlineStr">
+        <is>
+          <t>F29H85xMCAL_01.02.01: CDD ECAP - Automated Test Run</t>
+        </is>
+      </c>
+      <c r="S29" s="3" t="inlineStr"/>
+      <c r="T29" s="3" t="inlineStr"/>
+      <c r="U29" s="10" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:U27"/>
+  <autoFilter ref="A1:U29"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4008,12 +4746,12 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="12" t="inlineStr">
+      <c r="A2" s="11" t="inlineStr">
         <is>
           <t>Test Plan</t>
         </is>
       </c>
-      <c r="B2" s="13" t="inlineStr">
+      <c r="B2" s="12" t="inlineStr">
         <is>
           <t>Test Plan Key</t>
         </is>
@@ -4035,8 +4773,8 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="12" t="n"/>
-      <c r="B3" s="13" t="inlineStr">
+      <c r="A3" s="11" t="n"/>
+      <c r="B3" s="12" t="inlineStr">
         <is>
           <t>Test Plan Name</t>
         </is>
@@ -4058,8 +4796,8 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="12" t="n"/>
-      <c r="B4" s="13" t="inlineStr">
+      <c r="A4" s="11" t="n"/>
+      <c r="B4" s="12" t="inlineStr">
         <is>
           <t>Test Case Key</t>
         </is>
@@ -4081,8 +4819,8 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="12" t="n"/>
-      <c r="B5" s="13" t="inlineStr">
+      <c r="A5" s="11" t="n"/>
+      <c r="B5" s="12" t="inlineStr">
         <is>
           <t>Test Case Name</t>
         </is>
@@ -4104,8 +4842,8 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="12" t="n"/>
-      <c r="B6" s="13" t="inlineStr">
+      <c r="A6" s="11" t="n"/>
+      <c r="B6" s="12" t="inlineStr">
         <is>
           <t>Associated Issue(s) Type</t>
         </is>
@@ -4132,8 +4870,8 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="12" t="n"/>
-      <c r="B7" s="13" t="inlineStr">
+      <c r="A7" s="11" t="n"/>
+      <c r="B7" s="12" t="inlineStr">
         <is>
           <t>Associated Issue(s) ID(s)</t>
         </is>
@@ -4155,8 +4893,8 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="12" t="n"/>
-      <c r="B8" s="13" t="inlineStr">
+      <c r="A8" s="11" t="n"/>
+      <c r="B8" s="12" t="inlineStr">
         <is>
           <t>Test Platform</t>
         </is>
@@ -4178,8 +4916,8 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="12" t="n"/>
-      <c r="B9" s="13" t="inlineStr">
+      <c r="A9" s="11" t="n"/>
+      <c r="B9" s="12" t="inlineStr">
         <is>
           <t>Test Level</t>
         </is>
@@ -4195,7 +4933,7 @@
 -- "Not Provided" if no 'Test Scope' is provided in Jira</t>
         </is>
       </c>
-      <c r="D9" s="12" t="inlineStr">
+      <c r="D9" s="11" t="inlineStr">
         <is>
           <t>Optional</t>
         </is>
@@ -4207,8 +4945,8 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="12" t="n"/>
-      <c r="B10" s="13" t="inlineStr">
+      <c r="A10" s="11" t="n"/>
+      <c r="B10" s="12" t="inlineStr">
         <is>
           <t>Test Description</t>
         </is>
@@ -4230,8 +4968,8 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="12" t="n"/>
-      <c r="B11" s="13" t="inlineStr">
+      <c r="A11" s="11" t="n"/>
+      <c r="B11" s="12" t="inlineStr">
         <is>
           <t>Test Setup</t>
         </is>
@@ -4253,8 +4991,8 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="12" t="n"/>
-      <c r="B12" s="13" t="inlineStr">
+      <c r="A12" s="11" t="n"/>
+      <c r="B12" s="12" t="inlineStr">
         <is>
           <t>Pass/Fail Criteria</t>
         </is>
@@ -4276,8 +5014,8 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="12" t="n"/>
-      <c r="B13" s="13" t="inlineStr">
+      <c r="A13" s="11" t="n"/>
+      <c r="B13" s="12" t="inlineStr">
         <is>
           <t>Test Type</t>
         </is>
@@ -4288,7 +5026,7 @@
 (Map Test Method from Qmetry)</t>
         </is>
       </c>
-      <c r="D13" s="12" t="inlineStr">
+      <c r="D13" s="11" t="inlineStr">
         <is>
           <t>Optional</t>
         </is>
@@ -4300,15 +5038,15 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="12" t="n"/>
-      <c r="B14" s="13" t="n"/>
+      <c r="A14" s="11" t="n"/>
+      <c r="B14" s="12" t="n"/>
       <c r="C14" s="3" t="inlineStr">
         <is>
           <t>Functional:
 Tests covering functional requirements-based  aspects of the software</t>
         </is>
       </c>
-      <c r="D14" s="12" t="inlineStr">
+      <c r="D14" s="11" t="inlineStr">
         <is>
           <t>Optional</t>
         </is>
@@ -4320,8 +5058,8 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="12" t="n"/>
-      <c r="B15" s="13" t="n"/>
+      <c r="A15" s="11" t="n"/>
+      <c r="B15" s="12" t="n"/>
       <c r="C15" s="3" t="inlineStr">
         <is>
           <t>Compatability:
@@ -4329,7 +5067,7 @@
 ISO/IEC/IEEE 29119-1 Defn: type of testing that measures the degree to which a test item can function satisfactorily alongside other independent products in a shared environment (co-existence), and where necessary, exchanges information with other systems or components (interoperability)</t>
         </is>
       </c>
-      <c r="D15" s="12" t="inlineStr">
+      <c r="D15" s="11" t="inlineStr">
         <is>
           <t>Optional</t>
         </is>
@@ -4341,15 +5079,15 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="12" t="n"/>
-      <c r="B16" s="13" t="n"/>
+      <c r="A16" s="11" t="n"/>
+      <c r="B16" s="12" t="n"/>
       <c r="C16" s="3" t="inlineStr">
         <is>
           <t>Usability:
 Test Case covers usability/api/look and feel aspects of the module including out-of box (OOB) experience</t>
         </is>
       </c>
-      <c r="D16" s="12" t="inlineStr">
+      <c r="D16" s="11" t="inlineStr">
         <is>
           <t>Optional</t>
         </is>
@@ -4361,15 +5099,15 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="12" t="n"/>
-      <c r="B17" s="13" t="n"/>
+      <c r="A17" s="11" t="n"/>
+      <c r="B17" s="12" t="n"/>
       <c r="C17" s="3" t="inlineStr">
         <is>
           <t>Fault Injection:
 Testing based on injection of errors or faults to ensure no unintended consequences</t>
         </is>
       </c>
-      <c r="D17" s="12" t="inlineStr">
+      <c r="D17" s="11" t="inlineStr">
         <is>
           <t>Optional</t>
         </is>
@@ -4381,8 +5119,8 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="12" t="n"/>
-      <c r="B18" s="13" t="n"/>
+      <c r="A18" s="11" t="n"/>
+      <c r="B18" s="12" t="n"/>
       <c r="C18" s="3" t="inlineStr">
         <is>
           <t>Performance: 
@@ -4390,7 +5128,7 @@
 ISO/IEC/IEEE 29119-1 Defn: type of testing conducted to evaluate the degree to which a test item accomplishes its designated functions within given constraints of time and other resources</t>
         </is>
       </c>
-      <c r="D18" s="12" t="inlineStr">
+      <c r="D18" s="11" t="inlineStr">
         <is>
           <t>Optional</t>
         </is>
@@ -4402,8 +5140,8 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="12" t="n"/>
-      <c r="B19" s="13" t="n"/>
+      <c r="A19" s="11" t="n"/>
+      <c r="B19" s="12" t="n"/>
       <c r="C19" s="3" t="inlineStr">
         <is>
           <t>Reliability: 
@@ -4411,7 +5149,7 @@
 ISO/IEC/IEEE 29119-1 Defn: type of testing conducted to evaluate the ability of a test item to perform its required functions, including evaluating the frequency with which failures occur, when it is used under stated conditions for a specified period of time</t>
         </is>
       </c>
-      <c r="D19" s="12" t="inlineStr">
+      <c r="D19" s="11" t="inlineStr">
         <is>
           <t>Optional</t>
         </is>
@@ -4423,8 +5161,8 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="12" t="n"/>
-      <c r="B20" s="13" t="n"/>
+      <c r="A20" s="11" t="n"/>
+      <c r="B20" s="12" t="n"/>
       <c r="C20" s="3" t="inlineStr">
         <is>
           <t>Stress:
@@ -4432,7 +5170,7 @@
 ISO/IEC/IEEE 29119-1 Defn: type of performance efficiency testing conducted to evaluate a test item's behaviour under conditions of loading above anticipated or specified capacity requirements, or of resource availability below minimum specified requirements</t>
         </is>
       </c>
-      <c r="D20" s="12" t="inlineStr">
+      <c r="D20" s="11" t="inlineStr">
         <is>
           <t>Optional</t>
         </is>
@@ -4444,8 +5182,8 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="12" t="n"/>
-      <c r="B21" s="13" t="n"/>
+      <c r="A21" s="11" t="n"/>
+      <c r="B21" s="12" t="n"/>
       <c r="C21" s="3" t="inlineStr">
         <is>
           <t>Security:
@@ -4453,7 +5191,7 @@
 ISO/IEC/IEEE 29119-1 Defn: type of testing conducted to evaluate the degree to which a test item, and associated data and information, are protected so that unauthorized persons or systems cannot use, read, or modify them, and authorized persons or systems are not denied access to them</t>
         </is>
       </c>
-      <c r="D21" s="12" t="inlineStr">
+      <c r="D21" s="11" t="inlineStr">
         <is>
           <t>Optional</t>
         </is>
@@ -4465,8 +5203,8 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="12" t="n"/>
-      <c r="B22" s="13" t="n"/>
+      <c r="A22" s="11" t="n"/>
+      <c r="B22" s="12" t="n"/>
       <c r="C22" s="3" t="inlineStr">
         <is>
           <t>Maintainability:
@@ -4474,7 +5212,7 @@
 ISO/IEC/IEEE 29119-1 Defn: test type conducted to evaluate the degree of effectiveness and efficiency with which a test item may be modified</t>
         </is>
       </c>
-      <c r="D22" s="12" t="inlineStr">
+      <c r="D22" s="11" t="inlineStr">
         <is>
           <t>Optional</t>
         </is>
@@ -4486,8 +5224,8 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="12" t="n"/>
-      <c r="B23" s="13" t="n"/>
+      <c r="A23" s="11" t="n"/>
+      <c r="B23" s="12" t="n"/>
       <c r="C23" s="3" t="inlineStr">
         <is>
           <t>Portability:
@@ -4495,7 +5233,7 @@
 ISO/IEC/IEEE 29119-1 Defn: type of testing conducted to evaluate the ease with which a test item can be transferred from one hardware or software environment to another, including the level of modification needed for it to be executed in various types of environment</t>
         </is>
       </c>
-      <c r="D23" s="12" t="inlineStr">
+      <c r="D23" s="11" t="inlineStr">
         <is>
           <t>Optional</t>
         </is>
@@ -4507,8 +5245,8 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="12" t="n"/>
-      <c r="B24" s="13" t="inlineStr">
+      <c r="A24" s="11" t="n"/>
+      <c r="B24" s="12" t="inlineStr">
         <is>
           <t>Test Design Technique</t>
         </is>
@@ -4520,7 +5258,7 @@
 (Map Test Derivation Method from Qmetry)</t>
         </is>
       </c>
-      <c r="D24" s="12" t="inlineStr">
+      <c r="D24" s="11" t="inlineStr">
         <is>
           <t>Optional</t>
         </is>
@@ -4532,8 +5270,8 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="12" t="n"/>
-      <c r="B25" s="13" t="n"/>
+      <c r="A25" s="11" t="n"/>
+      <c r="B25" s="12" t="n"/>
       <c r="C25" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Requirements-Analysis:
@@ -4541,7 +5279,7 @@
 </t>
         </is>
       </c>
-      <c r="D25" s="12" t="inlineStr">
+      <c r="D25" s="11" t="inlineStr">
         <is>
           <t>Optional</t>
         </is>
@@ -4553,15 +5291,15 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="12" t="n"/>
-      <c r="B26" s="13" t="n"/>
+      <c r="A26" s="11" t="n"/>
+      <c r="B26" s="12" t="n"/>
       <c r="C26" s="3" t="inlineStr">
         <is>
           <t>Boundary Value Analysis:
 Test cases that apply to interfaces and values approaching and crossing the boundaries and out of range values</t>
         </is>
       </c>
-      <c r="D26" s="12" t="inlineStr">
+      <c r="D26" s="11" t="inlineStr">
         <is>
           <t>Optional</t>
         </is>
@@ -4573,15 +5311,15 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="12" t="n"/>
-      <c r="B27" s="13" t="n"/>
+      <c r="A27" s="11" t="n"/>
+      <c r="B27" s="12" t="n"/>
       <c r="C27" s="3" t="inlineStr">
         <is>
           <t>Error Guessing:
 Test cases established based on lessons learned and expert judgement to determine situations that may cause software failures or errors to appear</t>
         </is>
       </c>
-      <c r="D27" s="12" t="inlineStr">
+      <c r="D27" s="11" t="inlineStr">
         <is>
           <t>Optional</t>
         </is>
@@ -4593,28 +5331,28 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="12" t="n"/>
-      <c r="B28" s="13" t="n"/>
+      <c r="A28" s="11" t="n"/>
+      <c r="B28" s="12" t="n"/>
       <c r="C28" s="3" t="inlineStr">
         <is>
           <t>Other (Use case analysis; Customer Usage; Requirement analysis; Failure Mode analysis):
 Teams are encouraged to use techniques defined by standards such as ISO/IEC/IEEE 29119-4; which needs to be refelcted within Qmetry</t>
         </is>
       </c>
-      <c r="D28" s="12" t="inlineStr">
+      <c r="D28" s="11" t="inlineStr">
         <is>
           <t>Optional</t>
         </is>
       </c>
-      <c r="E28" s="12" t="inlineStr">
+      <c r="E28" s="11" t="inlineStr">
         <is>
           <t>Optional</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="12" t="n"/>
-      <c r="B29" s="13" t="inlineStr">
+      <c r="A29" s="11" t="n"/>
+      <c r="B29" s="12" t="inlineStr">
         <is>
           <t>Test Execution Type</t>
         </is>
@@ -4624,7 +5362,7 @@
           <t>Identifies whether the case is automated or manually or Semi-Automated executed</t>
         </is>
       </c>
-      <c r="D29" s="12" t="inlineStr">
+      <c r="D29" s="11" t="inlineStr">
         <is>
           <t>Optional</t>
         </is>
@@ -4636,8 +5374,8 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="12" t="n"/>
-      <c r="B30" s="13" t="inlineStr">
+      <c r="A30" s="11" t="n"/>
+      <c r="B30" s="12" t="inlineStr">
         <is>
           <t>Test Category</t>
         </is>
@@ -4647,7 +5385,7 @@
           <t>Test Categories represent sets of tests that are commonly used.</t>
         </is>
       </c>
-      <c r="D30" s="12" t="inlineStr">
+      <c r="D30" s="11" t="inlineStr">
         <is>
           <t>Optional</t>
         </is>
@@ -4659,15 +5397,15 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="12" t="n"/>
-      <c r="B31" s="13" t="n"/>
+      <c r="A31" s="11" t="n"/>
+      <c r="B31" s="12" t="n"/>
       <c r="C31" s="3" t="inlineStr">
         <is>
           <t>Sanity:
 This Test case is identified to run for Sanity Checks. These are mainly the basic tests that need to be run as part of entry to validate phase</t>
         </is>
       </c>
-      <c r="D31" s="12" t="inlineStr">
+      <c r="D31" s="11" t="inlineStr">
         <is>
           <t>Optional</t>
         </is>
@@ -4679,15 +5417,15 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="12" t="n"/>
-      <c r="B32" s="13" t="n"/>
+      <c r="A32" s="11" t="n"/>
+      <c r="B32" s="12" t="n"/>
       <c r="C32" s="3" t="inlineStr">
         <is>
           <t>Full:
 This category means running all test cases for identified releases</t>
         </is>
       </c>
-      <c r="D32" s="12" t="inlineStr">
+      <c r="D32" s="11" t="inlineStr">
         <is>
           <t>Optional</t>
         </is>
@@ -4699,15 +5437,15 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="12" t="n"/>
-      <c r="B33" s="13" t="n"/>
+      <c r="A33" s="11" t="n"/>
+      <c r="B33" s="12" t="n"/>
       <c r="C33" s="3" t="inlineStr">
         <is>
           <t>Base Regression:
 This Test case is identified to run for the Base Regression / maintenance releases</t>
         </is>
       </c>
-      <c r="D33" s="12" t="inlineStr">
+      <c r="D33" s="11" t="inlineStr">
         <is>
           <t>Optional</t>
         </is>
@@ -4719,8 +5457,8 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="12" t="n"/>
-      <c r="B34" s="13" t="inlineStr">
+      <c r="A34" s="11" t="n"/>
+      <c r="B34" s="12" t="inlineStr">
         <is>
           <t>Test Component(s)</t>
         </is>
@@ -4730,24 +5468,24 @@
           <t xml:space="preserve">The field provides the Component(s) (in Jira) to which the Test Case is mapped to. </t>
         </is>
       </c>
-      <c r="D34" s="12" t="inlineStr">
+      <c r="D34" s="11" t="inlineStr">
         <is>
           <t>Optional</t>
         </is>
       </c>
-      <c r="E34" s="12" t="inlineStr">
+      <c r="E34" s="11" t="inlineStr">
         <is>
           <t>Optional</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="14" t="inlineStr">
+      <c r="A35" s="13" t="inlineStr">
         <is>
           <t>Test Execution</t>
         </is>
       </c>
-      <c r="B35" s="13" t="inlineStr">
+      <c r="B35" s="12" t="inlineStr">
         <is>
           <t>Build/Release Key</t>
         </is>
@@ -4769,8 +5507,8 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="14" t="n"/>
-      <c r="B36" s="13" t="inlineStr">
+      <c r="A36" s="13" t="n"/>
+      <c r="B36" s="12" t="inlineStr">
         <is>
           <t>Defect Key</t>
         </is>
@@ -4792,8 +5530,8 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="14" t="n"/>
-      <c r="B37" s="13" t="inlineStr">
+      <c r="A37" s="13" t="n"/>
+      <c r="B37" s="12" t="inlineStr">
         <is>
           <t>Defect Summary</t>
         </is>
@@ -4815,8 +5553,8 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="14" t="n"/>
-      <c r="B38" s="13" t="inlineStr">
+      <c r="A38" s="13" t="n"/>
+      <c r="B38" s="12" t="inlineStr">
         <is>
           <t>Overall Status</t>
         </is>
@@ -4839,8 +5577,8 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="14" t="n"/>
-      <c r="B39" s="13" t="n"/>
+      <c r="A39" s="13" t="n"/>
+      <c r="B39" s="12" t="n"/>
       <c r="C39" s="3" t="inlineStr">
         <is>
           <t>PASS
@@ -4859,8 +5597,8 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="14" t="n"/>
-      <c r="B40" s="13" t="n"/>
+      <c r="A40" s="13" t="n"/>
+      <c r="B40" s="12" t="n"/>
       <c r="C40" s="3" t="inlineStr">
         <is>
           <t>FAIL
@@ -4879,8 +5617,8 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="14" t="n"/>
-      <c r="B41" s="13" t="n"/>
+      <c r="A41" s="13" t="n"/>
+      <c r="B41" s="12" t="n"/>
       <c r="C41" s="3" t="inlineStr">
         <is>
           <t>BLOCKED
@@ -4899,8 +5637,8 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="14" t="n"/>
-      <c r="B42" s="13" t="n"/>
+      <c r="A42" s="13" t="n"/>
+      <c r="B42" s="12" t="n"/>
       <c r="C42" s="3" t="inlineStr">
         <is>
           <t>WIP

</xml_diff>